<commit_message>
Temperatures, tilt sensor fault handling, board rev 2.7, drilling template
- Board rev 2.7 (162 x 134 mm): on-board DS18B20 box-air sensor (U11) and a
  latching Micro-Fit 3-pin TEMP PROBE header (J14) on the 1-Wire bus (GPIO 4)
- Dash: BOX HOT warning (50/65 C, 2 C hysteresis) and ambient readout for
  cab/outside probes (each or averaged); --temps lists the sensors
- Tilt sensor fault handling: missing/dead/nonsense sensor shows "--" instead
  of a made-up angle, re-initialises on its own, logs once
- Simulator: '-' unplugs the tilt sensor, '=' steps the box temperature
- Printable 1:1 drilling template (breakout-board/docs/mounting-template.pdf)
  with check rulers and Actual-size print preference

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bobcat-dash-BOM.xlsx
+++ b/bobcat-dash-BOM.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">BOM!$5:$5</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">BOM!$A$5:$K$92</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">BOM!$A$5:$K$97</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="263">
   <si>
     <t xml:space="preserve">Bobcat Digital Dash — Bill of Materials</t>
   </si>
@@ -440,7 +440,7 @@
     <t xml:space="preserve">Bare PCB</t>
   </si>
   <si>
-    <t xml:space="preserve">150 × 134 mm, 2 layers, 1.6 mm, 1 oz</t>
+    <t xml:space="preserve">162 × 134 mm (rev 2.7), 2 layers, 1.6 mm, 1 oz</t>
   </si>
   <si>
     <t xml:space="preserve">breakout-board/fab gerbers zip</t>
@@ -615,6 +615,39 @@
   </si>
   <si>
     <t xml:space="preserve">Subtotal — Machine Angle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEMPERATURE: README, Temperatures</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waterproof temperature probe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DS18B20 in a stainless tip, 3-wire cable (red 3V3, black GND, yellow/white data)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">README: Temperatures</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One for the cab, one for outside air (shade it from sun and engine heat). Optional: the board measures the box itself</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3-position, single row, latching</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Molex 43645-0300</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Board README: TEMP PROBE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plugs into the board's TEMP PROBE header J14 (43650-0315)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two probes: join their 3 wires in the cable (each wire to the same pin)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtotal — Temperature: Readme, Temperatures</t>
   </si>
   <si>
     <t xml:space="preserve">CHARGING: Delco 10SI 3-wire alternator (wiring-schematic.jpg, section 7)</t>
@@ -1434,7 +1467,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K97"/>
+  <dimension ref="A1:K102"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="6"/>
@@ -3215,12 +3248,12 @@
       <c r="J72" s="5"/>
       <c r="K72" s="5"/>
     </row>
-    <row r="73" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="6" t="n">
         <v>51</v>
       </c>
       <c r="B73" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C73" s="8" t="s">
         <v>198</v>
@@ -3229,13 +3262,13 @@
         <v>199</v>
       </c>
       <c r="E73" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F73" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="F73" s="6" t="s">
+      <c r="G73" s="8" t="s">
         <v>201</v>
-      </c>
-      <c r="G73" s="8" t="s">
-        <v>202</v>
       </c>
       <c r="H73" s="9"/>
       <c r="I73" s="10" t="n">
@@ -3253,16 +3286,16 @@
         <v>1</v>
       </c>
       <c r="C74" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="D74" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="E74" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="D74" s="8" t="s">
+      <c r="F74" s="6" t="s">
         <v>204</v>
-      </c>
-      <c r="E74" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F74" s="6" t="s">
-        <v>201</v>
       </c>
       <c r="G74" s="8" t="s">
         <v>205</v>
@@ -3275,27 +3308,27 @@
       <c r="J74" s="11"/>
       <c r="K74" s="12"/>
     </row>
-    <row r="75" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="6" t="n">
         <v>53</v>
       </c>
       <c r="B75" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C75" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="D75" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="E75" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="F75" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="G75" s="8" t="s">
         <v>206</v>
-      </c>
-      <c r="D75" s="8" t="s">
-        <v>207</v>
-      </c>
-      <c r="E75" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F75" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="G75" s="8" t="s">
-        <v>208</v>
       </c>
       <c r="H75" s="9"/>
       <c r="I75" s="10" t="n">
@@ -3307,7 +3340,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G76" s="13" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I76" s="14" t="n">
         <f aca="false">SUM(I73:I75)</f>
@@ -3316,7 +3349,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="5" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B77" s="5"/>
       <c r="C77" s="5"/>
@@ -3329,7 +3362,7 @@
       <c r="J77" s="5"/>
       <c r="K77" s="5"/>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="6" t="n">
         <v>54</v>
       </c>
@@ -3337,16 +3370,16 @@
         <v>1</v>
       </c>
       <c r="C78" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="D78" s="8" t="s">
+        <v>210</v>
+      </c>
+      <c r="E78" s="8" t="s">
         <v>211</v>
       </c>
-      <c r="D78" s="8" t="s">
+      <c r="F78" s="6" t="s">
         <v>212</v>
-      </c>
-      <c r="E78" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F78" s="6" t="s">
-        <v>23</v>
       </c>
       <c r="G78" s="8" t="s">
         <v>213</v>
@@ -3359,7 +3392,7 @@
       <c r="J78" s="11"/>
       <c r="K78" s="12"/>
     </row>
-    <row r="79" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="6" t="n">
         <v>55</v>
       </c>
@@ -3376,7 +3409,7 @@
         <v>23</v>
       </c>
       <c r="F79" s="6" t="s">
-        <v>23</v>
+        <v>212</v>
       </c>
       <c r="G79" s="8" t="s">
         <v>216</v>
@@ -3389,7 +3422,7 @@
       <c r="J79" s="11"/>
       <c r="K79" s="12"/>
     </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="6" t="n">
         <v>56</v>
       </c>
@@ -3406,7 +3439,7 @@
         <v>23</v>
       </c>
       <c r="F80" s="6" t="s">
-        <v>23</v>
+        <v>212</v>
       </c>
       <c r="G80" s="8" t="s">
         <v>219</v>
@@ -3420,77 +3453,41 @@
       <c r="K80" s="12"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="6" t="n">
-        <v>57</v>
-      </c>
-      <c r="B81" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C81" s="8" t="s">
+      <c r="G81" s="13" t="s">
         <v>220</v>
       </c>
-      <c r="D81" s="8" t="s">
+      <c r="I81" s="14" t="n">
+        <f aca="false">SUM(I78:I80)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="E81" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F81" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="G81" s="8" t="s">
-        <v>222</v>
-      </c>
-      <c r="H81" s="9"/>
-      <c r="I81" s="10" t="n">
-        <f aca="false">B81*H81</f>
-        <v>0</v>
-      </c>
-      <c r="J81" s="11"/>
-      <c r="K81" s="12"/>
-    </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="6" t="n">
-        <v>58</v>
-      </c>
-      <c r="B82" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C82" s="8" t="s">
-        <v>223</v>
-      </c>
-      <c r="D82" s="8" t="s">
-        <v>224</v>
-      </c>
-      <c r="E82" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F82" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="G82" s="8" t="s">
-        <v>225</v>
-      </c>
-      <c r="H82" s="9"/>
-      <c r="I82" s="10" t="n">
-        <f aca="false">B82*H82</f>
-        <v>0</v>
-      </c>
-      <c r="J82" s="11"/>
-      <c r="K82" s="12"/>
+      <c r="B82" s="5"/>
+      <c r="C82" s="5"/>
+      <c r="D82" s="5"/>
+      <c r="E82" s="5"/>
+      <c r="F82" s="5"/>
+      <c r="G82" s="5"/>
+      <c r="H82" s="5"/>
+      <c r="I82" s="5"/>
+      <c r="J82" s="5"/>
+      <c r="K82" s="5"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="6" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B83" s="7" t="n">
         <v>1</v>
       </c>
       <c r="C83" s="8" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="D83" s="8" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="E83" s="8" t="s">
         <v>23</v>
@@ -3499,7 +3496,7 @@
         <v>23</v>
       </c>
       <c r="G83" s="8" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="H83" s="9"/>
       <c r="I83" s="10" t="n">
@@ -3509,18 +3506,18 @@
       <c r="J83" s="11"/>
       <c r="K83" s="12"/>
     </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="6" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B84" s="7" t="n">
         <v>1</v>
       </c>
       <c r="C84" s="8" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D84" s="8" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E84" s="8" t="s">
         <v>23</v>
@@ -3529,7 +3526,7 @@
         <v>23</v>
       </c>
       <c r="G84" s="8" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="H84" s="9"/>
       <c r="I84" s="10" t="n">
@@ -3541,16 +3538,16 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="6" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B85" s="7" t="n">
         <v>1</v>
       </c>
       <c r="C85" s="8" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D85" s="8" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="E85" s="8" t="s">
         <v>23</v>
@@ -3559,7 +3556,7 @@
         <v>23</v>
       </c>
       <c r="G85" s="8" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="H85" s="9"/>
       <c r="I85" s="10" t="n">
@@ -3570,28 +3567,64 @@
       <c r="K85" s="12"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G86" s="13" t="s">
+      <c r="A86" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="B86" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C86" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="D86" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="E86" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F86" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="G86" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="H86" s="9"/>
+      <c r="I86" s="10" t="n">
+        <f aca="false">B86*H86</f>
+        <v>0</v>
+      </c>
+      <c r="J86" s="11"/>
+      <c r="K86" s="12"/>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="6" t="n">
+        <v>61</v>
+      </c>
+      <c r="B87" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C87" s="8" t="s">
         <v>234</v>
       </c>
-      <c r="I86" s="14" t="n">
-        <f aca="false">SUM(I78:I85)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="5" t="s">
+      <c r="D87" s="8" t="s">
         <v>235</v>
       </c>
-      <c r="B87" s="5"/>
-      <c r="C87" s="5"/>
-      <c r="D87" s="5"/>
-      <c r="E87" s="5"/>
-      <c r="F87" s="5"/>
-      <c r="G87" s="5"/>
-      <c r="H87" s="5"/>
-      <c r="I87" s="5"/>
-      <c r="J87" s="5"/>
-      <c r="K87" s="5"/>
+      <c r="E87" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F87" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="G87" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="H87" s="9"/>
+      <c r="I87" s="10" t="n">
+        <f aca="false">B87*H87</f>
+        <v>0</v>
+      </c>
+      <c r="J87" s="11"/>
+      <c r="K87" s="12"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="6" t="n">
@@ -3601,19 +3634,19 @@
         <v>1</v>
       </c>
       <c r="C88" s="8" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D88" s="8" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E88" s="8" t="s">
         <v>23</v>
       </c>
       <c r="F88" s="6" t="s">
-        <v>61</v>
+        <v>23</v>
       </c>
       <c r="G88" s="8" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="H88" s="9"/>
       <c r="I88" s="10" t="n">
@@ -3623,7 +3656,7 @@
       <c r="J88" s="11"/>
       <c r="K88" s="12"/>
     </row>
-    <row r="89" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="6" t="n">
         <v>63</v>
       </c>
@@ -3640,7 +3673,7 @@
         <v>23</v>
       </c>
       <c r="F89" s="6" t="s">
-        <v>61</v>
+        <v>23</v>
       </c>
       <c r="G89" s="8" t="s">
         <v>241</v>
@@ -3653,7 +3686,7 @@
       <c r="J89" s="11"/>
       <c r="K89" s="12"/>
     </row>
-    <row r="90" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="6" t="n">
         <v>64</v>
       </c>
@@ -3670,7 +3703,7 @@
         <v>23</v>
       </c>
       <c r="F90" s="6" t="s">
-        <v>61</v>
+        <v>23</v>
       </c>
       <c r="G90" s="8" t="s">
         <v>244</v>
@@ -3684,74 +3717,188 @@
       <c r="K90" s="12"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="6" t="n">
+      <c r="G91" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="I91" s="14" t="n">
+        <f aca="false">SUM(I83:I90)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="B92" s="5"/>
+      <c r="C92" s="5"/>
+      <c r="D92" s="5"/>
+      <c r="E92" s="5"/>
+      <c r="F92" s="5"/>
+      <c r="G92" s="5"/>
+      <c r="H92" s="5"/>
+      <c r="I92" s="5"/>
+      <c r="J92" s="5"/>
+      <c r="K92" s="5"/>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="6" t="n">
         <v>65</v>
       </c>
-      <c r="B91" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C91" s="8" t="s">
-        <v>245</v>
-      </c>
-      <c r="D91" s="8" t="s">
-        <v>246</v>
-      </c>
-      <c r="E91" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F91" s="6" t="s">
+      <c r="B93" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C93" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="D93" s="8" t="s">
+        <v>248</v>
+      </c>
+      <c r="E93" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F93" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="G93" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="H93" s="9"/>
+      <c r="I93" s="10" t="n">
+        <f aca="false">B93*H93</f>
+        <v>0</v>
+      </c>
+      <c r="J93" s="11"/>
+      <c r="K93" s="12"/>
+    </row>
+    <row r="94" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="6" t="n">
+        <v>66</v>
+      </c>
+      <c r="B94" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C94" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="D94" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="E94" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F94" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="G94" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="H94" s="9"/>
+      <c r="I94" s="10" t="n">
+        <f aca="false">B94*H94</f>
+        <v>0</v>
+      </c>
+      <c r="J94" s="11"/>
+      <c r="K94" s="12"/>
+    </row>
+    <row r="95" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="6" t="n">
+        <v>67</v>
+      </c>
+      <c r="B95" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C95" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="D95" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="E95" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F95" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="G95" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="H95" s="9"/>
+      <c r="I95" s="10" t="n">
+        <f aca="false">B95*H95</f>
+        <v>0</v>
+      </c>
+      <c r="J95" s="11"/>
+      <c r="K95" s="12"/>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="6" t="n">
+        <v>68</v>
+      </c>
+      <c r="B96" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C96" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="D96" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="E96" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F96" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="G91" s="8" t="s">
-        <v>247</v>
-      </c>
-      <c r="H91" s="9"/>
-      <c r="I91" s="10" t="n">
-        <f aca="false">B91*H91</f>
-        <v>0</v>
-      </c>
-      <c r="J91" s="11"/>
-      <c r="K91" s="12"/>
-    </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G92" s="13" t="s">
-        <v>248</v>
-      </c>
-      <c r="I92" s="14" t="n">
-        <f aca="false">SUM(I88:I91)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G94" s="15" t="s">
-        <v>249</v>
-      </c>
-      <c r="I94" s="16" t="n">
-        <f aca="false">I13+I19+I32+I38+I48+I56+I65+I71+I76+I86+I92</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G95" s="17" t="s">
-        <v>250</v>
-      </c>
-      <c r="I95" s="18" t="n">
-        <f aca="false">COUNTIF(B6:B86,"&gt;0")-COUNTIF(K6:K86,"Y")</f>
-        <v>58</v>
-      </c>
+      <c r="G96" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="H96" s="9"/>
+      <c r="I96" s="10" t="n">
+        <f aca="false">B96*H96</f>
+        <v>0</v>
+      </c>
+      <c r="J96" s="11"/>
+      <c r="K96" s="12"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="19" t="s">
-        <v>251</v>
+      <c r="G97" s="13" t="s">
+        <v>259</v>
+      </c>
+      <c r="I97" s="14" t="n">
+        <f aca="false">SUM(I93:I96)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G99" s="15" t="s">
+        <v>260</v>
+      </c>
+      <c r="I99" s="16" t="n">
+        <f aca="false">I13+I19+I32+I38+I48+I56+I65+I71+I76+I81+I91+I97</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G100" s="17" t="s">
+        <v>261</v>
+      </c>
+      <c r="I100" s="18" t="n">
+        <f aca="false">COUNTIF(B6:B91,"&gt;0")-COUNTIF(K6:K91,"Y")</f>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="19" t="s">
+        <v>262</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:K92"/>
+  <autoFilter ref="A5:K97"/>
   <mergeCells count="1">
     <mergeCell ref="A3:K3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K7:K12 K15:K18 K21:K31 K34:K37 K40:K47 K50:K55 K58:K64 K67:K70 K73:K75 K78:K85 K88:K91" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K7:K12 K15:K18 K21:K31 K34:K37 K40:K47 K50:K55 K58:K64 K67:K70 K73:K75 K78:K80 K83:K90 K93:K96" type="list">
       <formula1>"Y,N"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Board rev 2.8 re-layout: ribbon header on the top edge, amps side by side, 9 mounting holes, standoff keepouts
- Pi ribbon header J1 and the power LEDs move to the top edge (ribbon goes
  straight up to the lid); TILT plug to the top-left corner
- Stereo amp site J16 now sits beside the mono amp J9 ("fit one amp only")
- 9 M3 mounting holes against vibration: corners, mid-sides (H15-H18) and
  one near the centre (H19); drilling template updated
- Copper-free rings around every hole on both sides (M3 r 4 mm, M2.5 r 3 mm,
  extended to nearby edges): brass standoffs need no insulating washers and
  never tie board ground to the box
- ADS1115 adapter: same standoff keepouts
- README, parts list and BOM spreadsheet updated (9 M3 standoffs, brass notes)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bobcat-dash-BOM.xlsx
+++ b/bobcat-dash-BOM.xlsx
@@ -10,7 +10,7 @@
     <sheet name="BOM" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOM'!$A$5:$K$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOM'!$A$5:$K$100</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'BOM'!$5:$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K104"/>
+  <dimension ref="A1:K105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="G92" s="8" t="inlineStr">
         <is>
-          <t>Mount Pi and boards</t>
+          <t>Mount the Pi and the plug-in modules</t>
         </is>
       </c>
       <c r="H92" s="9" t="n"/>
@@ -3573,72 +3573,72 @@
       <c r="K92" s="12" t="n"/>
     </row>
     <row r="93">
-      <c r="G93" s="13" t="inlineStr">
+      <c r="A93" s="6" t="n">
+        <v>67</v>
+      </c>
+      <c r="B93" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="C93" s="8" t="inlineStr">
+        <is>
+          <t>M3 standoff + screws</t>
+        </is>
+      </c>
+      <c r="D93" s="8" t="inlineStr">
+        <is>
+          <t>10 mm or taller, all the same height</t>
+        </is>
+      </c>
+      <c r="E93" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F93" s="6" t="inlineStr">
+        <is>
+          <t>Board README</t>
+        </is>
+      </c>
+      <c r="G93" s="8" t="inlineStr">
+        <is>
+          <t>Breakout board mounting: 4 corners, 4 mid-sides, 1 centre (drilling template)</t>
+        </is>
+      </c>
+      <c r="H93" s="9" t="n"/>
+      <c r="I93" s="10">
+        <f>B93*H93</f>
+        <v/>
+      </c>
+      <c r="J93" s="11" t="n"/>
+      <c r="K93" s="12" t="n"/>
+    </row>
+    <row r="94">
+      <c r="G94" s="13" t="inlineStr">
         <is>
           <t>Subtotal — Wiring + Enclosure</t>
         </is>
       </c>
-      <c r="I93" s="14">
-        <f>SUM(I85:I92)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="5" t="inlineStr">
+      <c r="I94" s="14">
+        <f>SUM(I85:I93)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="inlineStr">
         <is>
           <t>EXISTING MACHINE PARTS (reuse, check they work)</t>
         </is>
       </c>
-      <c r="B94" s="5" t="n"/>
-      <c r="C94" s="5" t="n"/>
-      <c r="D94" s="5" t="n"/>
-      <c r="E94" s="5" t="n"/>
-      <c r="F94" s="5" t="n"/>
-      <c r="G94" s="5" t="n"/>
-      <c r="H94" s="5" t="n"/>
-      <c r="I94" s="5" t="n"/>
-      <c r="J94" s="5" t="n"/>
-      <c r="K94" s="5" t="n"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="6" t="n">
-        <v>67</v>
-      </c>
-      <c r="B95" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C95" s="8" t="inlineStr">
-        <is>
-          <t>Oil pressure switch</t>
-        </is>
-      </c>
-      <c r="D95" s="8" t="inlineStr">
-        <is>
-          <t>Original, closes on low pressure</t>
-        </is>
-      </c>
-      <c r="E95" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F95" s="6" t="inlineStr">
-        <is>
-          <t>Sch. 5</t>
-        </is>
-      </c>
-      <c r="G95" s="8" t="inlineStr">
-        <is>
-          <t>GPIO 22 via optocoupler</t>
-        </is>
-      </c>
-      <c r="H95" s="9" t="n"/>
-      <c r="I95" s="10">
-        <f>B95*H95</f>
-        <v/>
-      </c>
-      <c r="J95" s="11" t="n"/>
-      <c r="K95" s="12" t="n"/>
+      <c r="B95" s="5" t="n"/>
+      <c r="C95" s="5" t="n"/>
+      <c r="D95" s="5" t="n"/>
+      <c r="E95" s="5" t="n"/>
+      <c r="F95" s="5" t="n"/>
+      <c r="G95" s="5" t="n"/>
+      <c r="H95" s="5" t="n"/>
+      <c r="I95" s="5" t="n"/>
+      <c r="J95" s="5" t="n"/>
+      <c r="K95" s="5" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="6" t="n">
@@ -3649,12 +3649,12 @@
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t>Hydraulic filter bypass switch</t>
+          <t>Oil pressure switch</t>
         </is>
       </c>
       <c r="D96" s="8" t="inlineStr">
         <is>
-          <t>Original, closes on bypass</t>
+          <t>Original, closes on low pressure</t>
         </is>
       </c>
       <c r="E96" s="8" t="inlineStr">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="G96" s="8" t="inlineStr">
         <is>
-          <t>ADS1115 A2, monitored (4.7k EOL resistor at the switch)</t>
+          <t>GPIO 22 via optocoupler</t>
         </is>
       </c>
       <c r="H96" s="9" t="n"/>
@@ -3689,12 +3689,12 @@
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t>Hydraulic oil temp switch</t>
+          <t>Hydraulic filter bypass switch</t>
         </is>
       </c>
       <c r="D97" s="8" t="inlineStr">
         <is>
-          <t>Original, closes when hot</t>
+          <t>Original, closes on bypass</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
@@ -3709,7 +3709,7 @@
       </c>
       <c r="G97" s="8" t="inlineStr">
         <is>
-          <t>ADS1115 A3, monitored (4.7k EOL resistor at the switch)</t>
+          <t>ADS1115 A2, monitored (4.7k EOL resistor at the switch)</t>
         </is>
       </c>
       <c r="H97" s="9" t="n"/>
@@ -3729,12 +3729,12 @@
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t>Fuel sender</t>
+          <t>Hydraulic oil temp switch</t>
         </is>
       </c>
       <c r="D98" s="8" t="inlineStr">
         <is>
-          <t>Original, in tank</t>
+          <t>Original, closes when hot</t>
         </is>
       </c>
       <c r="E98" s="8" t="inlineStr">
@@ -3744,12 +3744,12 @@
       </c>
       <c r="F98" s="6" t="inlineStr">
         <is>
-          <t>Sch. 4</t>
+          <t>Sch. 5</t>
         </is>
       </c>
       <c r="G98" s="8" t="inlineStr">
         <is>
-          <t>Calibrate with dash.py --calibrate</t>
+          <t>ADS1115 A3, monitored (4.7k EOL resistor at the switch)</t>
         </is>
       </c>
       <c r="H98" s="9" t="n"/>
@@ -3761,52 +3761,92 @@
       <c r="K98" s="12" t="n"/>
     </row>
     <row r="99">
-      <c r="G99" s="13" t="inlineStr">
+      <c r="A99" s="6" t="n">
+        <v>71</v>
+      </c>
+      <c r="B99" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C99" s="8" t="inlineStr">
+        <is>
+          <t>Fuel sender</t>
+        </is>
+      </c>
+      <c r="D99" s="8" t="inlineStr">
+        <is>
+          <t>Original, in tank</t>
+        </is>
+      </c>
+      <c r="E99" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F99" s="6" t="inlineStr">
+        <is>
+          <t>Sch. 4</t>
+        </is>
+      </c>
+      <c r="G99" s="8" t="inlineStr">
+        <is>
+          <t>Calibrate with dash.py --calibrate</t>
+        </is>
+      </c>
+      <c r="H99" s="9" t="n"/>
+      <c r="I99" s="10">
+        <f>B99*H99</f>
+        <v/>
+      </c>
+      <c r="J99" s="11" t="n"/>
+      <c r="K99" s="12" t="n"/>
+    </row>
+    <row r="100">
+      <c r="G100" s="13" t="inlineStr">
         <is>
           <t>Subtotal — Existing Machine Parts</t>
         </is>
       </c>
-      <c r="I99" s="14">
-        <f>SUM(I95:I98)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="101">
-      <c r="G101" s="15" t="inlineStr">
+      <c r="I100" s="14">
+        <f>SUM(I96:I99)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="G102" s="15" t="inlineStr">
         <is>
           <t>TOTAL (all sections)</t>
         </is>
       </c>
-      <c r="I101" s="16">
-        <f>I13+I19+I33+I39+I50+I58+I67+I73+I78+I83+I93+I99</f>
-        <v/>
-      </c>
-    </row>
-    <row r="102">
-      <c r="G102" s="17" t="inlineStr">
+      <c r="I102" s="16">
+        <f>I13+I19+I33+I39+I50+I58+I67+I73+I78+I83+I94+I100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="G103" s="17" t="inlineStr">
         <is>
           <t>Items still to order (excl. existing parts)</t>
         </is>
       </c>
-      <c r="I102" s="18">
-        <f>COUNTIF(B6:B93,"&gt;0")-COUNTIF(K6:K93,"Y")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="19" t="inlineStr">
+      <c r="I103" s="18">
+        <f>COUNTIF(B6:B94,"&gt;0")-COUNTIF(K6:K94,"Y")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="19" t="inlineStr">
         <is>
           <t>Notes: Qty in blue = quantity per machine. Existing machine parts usually cost $0 unless one needs replacing. Prices are left blank on purpose. Enter what you actually pay.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:K99"/>
+  <autoFilter ref="A5:K100"/>
   <mergeCells count="1">
     <mergeCell ref="A3:K3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="K7 K8 K9 K10 K11 K12 K15 K16 K17 K18 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K35 K36 K37 K38 K41 K42 K43 K44 K45 K46 K47 K48 K49 K52 K53 K54 K55 K56 K57 K60 K61 K62 K63 K64 K65 K66 K69 K70 K71 K72 K75 K76 K77 K80 K81 K82 K85 K86 K87 K88 K89 K90 K91 K92 K95 K96 K97 K98" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K7 K8 K9 K10 K11 K12 K15 K16 K17 K18 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K35 K36 K37 K38 K41 K42 K43 K44 K45 K46 K47 K48 K49 K52 K53 K54 K55 K56 K57 K60 K61 K62 K63 K64 K65 K66 K69 K70 K71 K72 K75 K76 K77 K80 K81 K82 K85 K86 K87 K88 K89 K90 K91 K92 K93 K96 K97 K98 K99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>